<commit_message>
ST:lab6 modified. Lab7 done(some tests fail but still:) )
</commit_message>
<xml_diff>
--- a/ST/Reports/Lab_6/Lab_6.xlsx
+++ b/ST/Reports/Lab_6/Lab_6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manmade\Desktop\6sem\ST\Reports\Lab_6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4674F05C-350D-4C84-80C8-ABB219359CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D4E72B-3E81-480B-A042-FEDA233D3325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
     <t>Сценарий 1: Создание задачи через панель проекта</t>
   </si>
   <si>
-    <t>[Главная] → [Список проектов] → [Проект] → [Доска Kanban] → [Создать задачу] → [Форма задачи] → [Сохранить] → [Задача на доске ★]</t>
-  </si>
-  <si>
     <t>Шаг</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>Сценарий 2: Создание задачи через быстрое добавление из бэклога</t>
   </si>
   <si>
-    <t>[Главная] → [Навигация] → [Бэклог] → [Быстрое добавление] → [Ввод названия] → [Выбор проекта] → [Назначение спринта] → [Сохранить] → [Задача в бэклоге ★]</t>
-  </si>
-  <si>
     <t>В меню навигации выбрать раздел "Бэклог"</t>
   </si>
   <si>
@@ -160,9 +154,6 @@
   </si>
   <si>
     <t>Сценарий 3: Создание задачи через дублирование существующей</t>
-  </si>
-  <si>
-    <t>[Главная] → [Поиск задачи] → [Просмотр задачи] → [Дублировать] → [Редактирование полей] → [Изменение исполнителя/дедлайна] → [Сохранить] → [Новая задача ★]</t>
   </si>
   <si>
     <t>Воспользоваться строкой поиска для нахождения существующей задачи</t>
@@ -459,6 +450,15 @@
   </si>
   <si>
     <t>В фокусе внимания — устойчивость и безопасность системы. Проверяется обработка ошибок, валидация входных данных, защита от SQL-инъекций и XSS-атак, поведение системы при граничных значениях и стрессовых условиях. Диверсант выявляет уязвимости и сценарии, способные привести к сбоям, потере данных или нарушению безопасности. Особое внимание уделяется тому, насколько система информирует пользователя о недопустимых действиях.</t>
+  </si>
+  <si>
+    <t>[Главная] → [Список проектов] → [Проект] → [Доска Kanban] → [Создать задачу] → [Форма задачи] → [Сохранить] → [Задача на доске ]</t>
+  </si>
+  <si>
+    <t>[Главная] → [Навигация] → [Бэклог] → [Быстрое добавление] → [Ввод названия] → [Выбор проекта] → [Назначение спринта] → [Сохранить] → [Задача в бэклоге]</t>
+  </si>
+  <si>
+    <t>[Главная] → [Поиск задачи] → [Просмотр задачи] → [Дублировать] → [Редактирование полей] → [Изменение исполнителя/дедлайна] → [Сохранить] → [Новая задача]</t>
   </si>
 </sst>
 </file>
@@ -582,17 +582,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -916,334 +916,334 @@
     </row>
     <row r="2" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>30</v>
+        <v>141</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
     </row>
     <row r="26" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>46</v>
+        <v>142</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B34" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="C34" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1269,199 +1269,207 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="10"/>
+      <c r="A1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="10"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B9" s="12"/>
+    </row>
+    <row r="10" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="B10" s="12"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="12"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="9"/>
-    </row>
-    <row r="10" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="B12" s="12"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="10"/>
+    </row>
+    <row r="14" spans="1:2" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="9"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="B14" s="12"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="9"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="9"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="12"/>
-    </row>
-    <row r="14" spans="1:2" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="9"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" s="10"/>
+      <c r="B16" s="8"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="10"/>
+    </row>
+    <row r="24" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="12"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="12"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" s="12"/>
-    </row>
-    <row r="24" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
+      <c r="B26" s="12"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="B24" s="9"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
+      <c r="B27" s="12"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="10"/>
+    </row>
+    <row r="29" spans="1:2" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="9"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="9"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B27" s="9"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" s="12"/>
-    </row>
-    <row r="29" spans="1:2" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B29" s="9"/>
+      <c r="B29" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A9:B9"/>
@@ -1470,14 +1478,6 @@
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1494,354 +1494,380 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B1" s="14"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="12"/>
+    </row>
+    <row r="8" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="12"/>
+    </row>
+    <row r="9" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="B6" s="12"/>
-    </row>
-    <row r="7" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="B9" s="12"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="9"/>
-    </row>
-    <row r="8" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="B10" s="12"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="9"/>
-    </row>
-    <row r="9" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="B11" s="12"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="9"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="B12" s="12"/>
+    </row>
+    <row r="13" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="9"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="B13" s="12"/>
+    </row>
+    <row r="14" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="9"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="B14" s="12"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B12" s="9"/>
-    </row>
-    <row r="13" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="B15" s="12"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="B13" s="9"/>
-    </row>
-    <row r="14" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="9"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B15" s="9"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B16" s="9"/>
+      <c r="B16" s="12"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B17" s="12"/>
+        <v>106</v>
+      </c>
+      <c r="B17" s="10"/>
     </row>
     <row r="18" spans="1:2" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B18" s="9"/>
+      <c r="A18" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="12"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="12"/>
+        <v>95</v>
+      </c>
+      <c r="B25" s="10"/>
     </row>
     <row r="26" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B26" s="12"/>
+    </row>
+    <row r="27" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="12"/>
+    </row>
+    <row r="28" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="12"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="B26" s="9"/>
-    </row>
-    <row r="27" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+      <c r="B29" s="12"/>
+    </row>
+    <row r="30" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="B27" s="9"/>
-    </row>
-    <row r="28" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
+      <c r="B30" s="12"/>
+    </row>
+    <row r="31" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="B28" s="9"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
+      <c r="B31" s="12"/>
+    </row>
+    <row r="32" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="B29" s="9"/>
-    </row>
-    <row r="30" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
+      <c r="B32" s="12"/>
+    </row>
+    <row r="33" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="B30" s="9"/>
-    </row>
-    <row r="31" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
+      <c r="B33" s="12"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="9"/>
-    </row>
-    <row r="32" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
+      <c r="B34" s="12"/>
+    </row>
+    <row r="35" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="B32" s="9"/>
-    </row>
-    <row r="33" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B33" s="9"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B34" s="9"/>
-    </row>
-    <row r="35" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B35" s="9"/>
+      <c r="B35" s="12"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B36" s="12"/>
+        <v>106</v>
+      </c>
+      <c r="B36" s="10"/>
     </row>
     <row r="37" spans="1:2" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B37" s="9"/>
+      <c r="A37" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B37" s="12"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B39" s="14"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="B44" s="12"/>
+        <v>95</v>
+      </c>
+      <c r="B44" s="10"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B45" s="12"/>
+    </row>
+    <row r="46" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="12"/>
+    </row>
+    <row r="47" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="12"/>
+    </row>
+    <row r="48" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="9"/>
-    </row>
-    <row r="46" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="8" t="s">
+      <c r="B48" s="12"/>
+    </row>
+    <row r="49" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="9"/>
-    </row>
-    <row r="47" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="8" t="s">
+      <c r="B49" s="12"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="9"/>
-    </row>
-    <row r="48" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="8" t="s">
+      <c r="B50" s="12"/>
+    </row>
+    <row r="51" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B48" s="9"/>
-    </row>
-    <row r="49" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8" t="s">
+      <c r="B51" s="12"/>
+    </row>
+    <row r="52" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="B49" s="9"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="8" t="s">
+      <c r="B52" s="12"/>
+    </row>
+    <row r="53" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B50" s="9"/>
-    </row>
-    <row r="51" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="8" t="s">
+      <c r="B53" s="12"/>
+    </row>
+    <row r="54" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="B51" s="9"/>
-    </row>
-    <row r="52" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B52" s="9"/>
-    </row>
-    <row r="53" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B53" s="9"/>
-    </row>
-    <row r="54" spans="1:2" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B54" s="9"/>
+      <c r="B54" s="12"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B55" s="12"/>
+        <v>106</v>
+      </c>
+      <c r="B55" s="10"/>
     </row>
     <row r="56" spans="1:2" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="B56" s="9"/>
+      <c r="A56" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B56" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A51:B51"/>
     <mergeCell ref="A56:B56"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="A12:B12"/>
@@ -1858,32 +1884,6 @@
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A49:B49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>